<commit_message>
Updated workbook and used different features
</commit_message>
<xml_diff>
--- a/week-01/Ex4A_GTrends.xlsx
+++ b/week-01/Ex4A_GTrends.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sultansimsek/Documents/DataAnalytics/week-01/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{175E9D04-9F76-3F4A-A597-99513FBF417A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF6B8693-FC79-0348-9D3C-A5D651205306}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14280" yWindow="760" windowWidth="15960" windowHeight="17140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1 - multiTimeline" sheetId="1" r:id="rId1"/>

</xml_diff>